<commit_message>
tampil pakai db depan
</commit_message>
<xml_diff>
--- a/db_dp3m_concept.xlsx
+++ b/db_dp3m_concept.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\dp3m.unsri\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44911604-E429-4A16-A9FB-E61C48A2C488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C284E8D-B11D-482F-BF88-F102A574A6C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="5" xr2:uid="{CCCD2181-656E-4380-A768-DEEB759A9327}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{CCCD2181-656E-4380-A768-DEEB759A9327}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="6_peraturan_dokumen" sheetId="1" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -395,9 +394,6 @@
     <t>strategis</t>
   </si>
   <si>
-    <t>Visi, Misi, Tujuan, dan Strategi DP3M</t>
-  </si>
-  <si>
     <t>Struktur Organisasi</t>
   </si>
   <si>
@@ -531,13 +527,16 @@
   </si>
   <si>
     <t>home_konten_text-short</t>
+  </si>
+  <si>
+    <t>sekapur sirih</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -558,8 +557,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -570,6 +576,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -597,21 +608,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -954,12 +969,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="A1" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -977,16 +992,16 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" t="s">
         <v>124</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>125</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>126</v>
-      </c>
-      <c r="D3" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1000,7 +1015,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1014,7 +1029,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1028,7 +1043,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1042,7 +1057,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -1071,43 +1086,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="A1" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
         <v>124</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>125</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>126</v>
-      </c>
-      <c r="D2" t="s">
-        <v>127</v>
       </c>
       <c r="E2" t="s">
         <v>101</v>
       </c>
       <c r="F2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G2" t="s">
         <v>102</v>
       </c>
       <c r="H2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -1121,14 +1136,14 @@
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E3" t="str">
         <f>A3&amp;B3&amp;C3&amp;D3</f>
         <v>1010001</v>
       </c>
       <c r="F3" t="str">
-        <f>A3&amp;B3&amp;C3</f>
+        <f t="shared" ref="F3:F16" si="0">A3&amp;B3&amp;C3</f>
         <v>101</v>
       </c>
       <c r="G3" t="s">
@@ -1155,14 +1170,14 @@
         <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E4" t="str">
-        <f t="shared" ref="E4:E16" si="0">A4&amp;B4&amp;C4&amp;D4</f>
+        <f t="shared" ref="E4:E16" si="1">A4&amp;B4&amp;C4&amp;D4</f>
         <v>1020001</v>
       </c>
       <c r="F4" t="str">
-        <f>A4&amp;B4&amp;C4</f>
+        <f t="shared" si="0"/>
         <v>102</v>
       </c>
       <c r="G4" t="s">
@@ -1189,14 +1204,14 @@
         <v>2</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1020002</v>
       </c>
       <c r="F5" t="str">
-        <f>A5&amp;B5&amp;C5</f>
+        <f t="shared" si="0"/>
         <v>102</v>
       </c>
       <c r="G5" t="s">
@@ -1223,14 +1238,14 @@
         <v>2</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1020003</v>
       </c>
       <c r="F6" t="str">
-        <f>A6&amp;B6&amp;C6</f>
+        <f t="shared" si="0"/>
         <v>102</v>
       </c>
       <c r="G6" t="s">
@@ -1246,343 +1261,343 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7">
+    <row r="7" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>1</v>
+      </c>
+      <c r="B7" s="4">
         <v>0</v>
       </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="C7" s="4">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E7" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1030001</v>
+      </c>
+      <c r="F7" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>103</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>1</v>
+      </c>
+      <c r="B8" s="4">
+        <v>0</v>
+      </c>
+      <c r="C8" s="4">
+        <v>4</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1040001</v>
+      </c>
+      <c r="F8" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>104</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>1</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0</v>
+      </c>
+      <c r="C9" s="4">
+        <v>5</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E9" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1050001</v>
+      </c>
+      <c r="F9" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>105</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>1</v>
+      </c>
+      <c r="B10" s="4">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4">
+        <v>5</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E7" t="str">
-        <f t="shared" si="0"/>
-        <v>1030001</v>
-      </c>
-      <c r="F7" t="str">
-        <f>A7&amp;B7&amp;C7</f>
-        <v>103</v>
-      </c>
-      <c r="G7" t="s">
-        <v>99</v>
-      </c>
-      <c r="H7" t="s">
-        <v>48</v>
-      </c>
-      <c r="I7" t="s">
-        <v>159</v>
-      </c>
-      <c r="J7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8">
+      <c r="E10" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1050002</v>
+      </c>
+      <c r="F10" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>105</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>1</v>
+      </c>
+      <c r="B11" s="4">
         <v>0</v>
       </c>
-      <c r="C8">
-        <v>4</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="C11" s="4">
+        <v>5</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1050003</v>
+      </c>
+      <c r="F11" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>105</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>1</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4">
+        <v>6</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E12" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1060001</v>
+      </c>
+      <c r="F12" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>106</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>1</v>
+      </c>
+      <c r="B13" s="4">
+        <v>0</v>
+      </c>
+      <c r="C13" s="4">
+        <v>6</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E8" t="str">
-        <f t="shared" si="0"/>
-        <v>1040001</v>
-      </c>
-      <c r="F8" t="str">
-        <f>A8&amp;B8&amp;C8</f>
-        <v>104</v>
-      </c>
-      <c r="G8" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I8" t="s">
-        <v>48</v>
-      </c>
-      <c r="J8" t="s">
+      <c r="E13" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1060002</v>
+      </c>
+      <c r="F13" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>106</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J13" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>1</v>
-      </c>
-      <c r="B9">
+    <row r="14" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>1</v>
+      </c>
+      <c r="B14" s="4">
         <v>0</v>
       </c>
-      <c r="C9">
-        <v>5</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E9" t="str">
-        <f t="shared" si="0"/>
-        <v>1050001</v>
-      </c>
-      <c r="F9" t="str">
-        <f>A9&amp;B9&amp;C9</f>
-        <v>105</v>
-      </c>
-      <c r="G9" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" t="s">
-        <v>48</v>
-      </c>
-      <c r="I9" t="s">
-        <v>48</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="C14" s="4">
+        <v>6</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E14" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1060003</v>
+      </c>
+      <c r="F14" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>106</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J14" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>1</v>
-      </c>
-      <c r="B10">
+    <row r="15" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>1</v>
+      </c>
+      <c r="B15" s="4">
         <v>0</v>
       </c>
-      <c r="C10">
-        <v>5</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E10" t="str">
-        <f t="shared" si="0"/>
-        <v>1050002</v>
-      </c>
-      <c r="F10" t="str">
-        <f>A10&amp;B10&amp;C10</f>
-        <v>105</v>
-      </c>
-      <c r="G10" t="s">
-        <v>48</v>
-      </c>
-      <c r="H10" t="s">
-        <v>48</v>
-      </c>
-      <c r="I10" t="s">
-        <v>48</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="C15" s="4">
+        <v>6</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1060004</v>
+      </c>
+      <c r="F15" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>106</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11">
+    <row r="16" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>1</v>
+      </c>
+      <c r="B16" s="4">
         <v>0</v>
       </c>
-      <c r="C11">
-        <v>5</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E11" t="str">
-        <f t="shared" si="0"/>
-        <v>1050003</v>
-      </c>
-      <c r="F11" t="str">
-        <f>A11&amp;B11&amp;C11</f>
-        <v>105</v>
-      </c>
-      <c r="G11" t="s">
-        <v>48</v>
-      </c>
-      <c r="H11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11" t="s">
-        <v>48</v>
-      </c>
-      <c r="J11" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>1</v>
-      </c>
-      <c r="B12">
-        <v>0</v>
-      </c>
-      <c r="C12">
+      <c r="C16" s="4">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E12" t="str">
-        <f t="shared" si="0"/>
-        <v>1060001</v>
-      </c>
-      <c r="F12" t="str">
-        <f>A12&amp;B12&amp;C12</f>
+      <c r="D16" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="E16" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>1060005</v>
+      </c>
+      <c r="F16" s="4" t="str">
+        <f t="shared" si="0"/>
         <v>106</v>
       </c>
-      <c r="G12" t="s">
-        <v>48</v>
-      </c>
-      <c r="H12" t="s">
-        <v>48</v>
-      </c>
-      <c r="I12" t="s">
-        <v>48</v>
-      </c>
-      <c r="J12" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>1</v>
-      </c>
-      <c r="B13">
-        <v>0</v>
-      </c>
-      <c r="C13">
-        <v>6</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E13" t="str">
-        <f t="shared" si="0"/>
-        <v>1060002</v>
-      </c>
-      <c r="F13" t="str">
-        <f>A13&amp;B13&amp;C13</f>
-        <v>106</v>
-      </c>
-      <c r="G13" t="s">
-        <v>48</v>
-      </c>
-      <c r="H13" t="s">
-        <v>48</v>
-      </c>
-      <c r="I13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J13" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>1</v>
-      </c>
-      <c r="B14">
-        <v>0</v>
-      </c>
-      <c r="C14">
-        <v>6</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E14" t="str">
-        <f t="shared" si="0"/>
-        <v>1060003</v>
-      </c>
-      <c r="F14" t="str">
-        <f>A14&amp;B14&amp;C14</f>
-        <v>106</v>
-      </c>
-      <c r="G14" t="s">
-        <v>48</v>
-      </c>
-      <c r="H14" t="s">
-        <v>48</v>
-      </c>
-      <c r="I14" t="s">
-        <v>48</v>
-      </c>
-      <c r="J14" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>1</v>
-      </c>
-      <c r="B15">
-        <v>0</v>
-      </c>
-      <c r="C15">
-        <v>6</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E15" t="str">
-        <f t="shared" si="0"/>
-        <v>1060004</v>
-      </c>
-      <c r="F15" t="str">
-        <f>A15&amp;B15&amp;C15</f>
-        <v>106</v>
-      </c>
-      <c r="G15" t="s">
-        <v>48</v>
-      </c>
-      <c r="H15" t="s">
-        <v>48</v>
-      </c>
-      <c r="I15" t="s">
-        <v>48</v>
-      </c>
-      <c r="J15" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>1</v>
-      </c>
-      <c r="B16">
-        <v>0</v>
-      </c>
-      <c r="C16">
-        <v>6</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="E16" t="str">
-        <f t="shared" si="0"/>
-        <v>1060005</v>
-      </c>
-      <c r="F16" t="str">
-        <f>A16&amp;B16&amp;C16</f>
-        <v>106</v>
-      </c>
-      <c r="G16" t="s">
-        <v>48</v>
-      </c>
-      <c r="H16" t="s">
-        <v>48</v>
-      </c>
-      <c r="I16" t="s">
-        <v>48</v>
-      </c>
-      <c r="J16" t="s">
+      <c r="G16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J16" s="4" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1612,226 +1627,226 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="A1" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
         <v>124</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>125</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>126</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="E2" t="s">
-        <v>118</v>
-      </c>
-      <c r="F2" t="s">
-        <v>146</v>
-      </c>
-      <c r="G2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E3" t="str">
+      <c r="E3" s="4" t="str">
         <f>A3&amp;B3&amp;C3&amp;D3</f>
         <v>2110001</v>
       </c>
-      <c r="F3" t="str">
-        <f>A3&amp;B3&amp;C3</f>
+      <c r="F3" s="4" t="str">
+        <f t="shared" ref="F3:F8" si="0">A3&amp;B3&amp;C3</f>
         <v>211</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E4" s="4" t="str">
+        <f t="shared" ref="E4:E8" si="1">A4&amp;B4&amp;C4&amp;D4</f>
+        <v>2120001</v>
+      </c>
+      <c r="F4" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>212</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4">
+        <v>3</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>2130001</v>
+      </c>
+      <c r="F5" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>213</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4">
+        <v>4</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E6" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>2140001</v>
+      </c>
+      <c r="F6" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>214</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>2</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4">
+        <v>5</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E7" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>2150001</v>
+      </c>
+      <c r="F7" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>215</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>2</v>
+      </c>
+      <c r="B8" s="4">
+        <v>2</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>2210001</v>
+      </c>
+      <c r="F8" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>221</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="H3" t="s">
-        <v>159</v>
-      </c>
-      <c r="I3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E4" t="str">
-        <f t="shared" ref="E4:E8" si="0">A4&amp;B4&amp;C4&amp;D4</f>
-        <v>2120001</v>
-      </c>
-      <c r="F4" t="str">
-        <f>A4&amp;B4&amp;C4</f>
-        <v>212</v>
-      </c>
-      <c r="G4" t="s">
-        <v>112</v>
-      </c>
-      <c r="H4" t="s">
-        <v>159</v>
-      </c>
-      <c r="I4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E5" t="str">
-        <f t="shared" si="0"/>
-        <v>2130001</v>
-      </c>
-      <c r="F5" t="str">
-        <f>A5&amp;B5&amp;C5</f>
-        <v>213</v>
-      </c>
-      <c r="G5" t="s">
-        <v>113</v>
-      </c>
-      <c r="H5" t="s">
-        <v>159</v>
-      </c>
-      <c r="I5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>4</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E6" t="str">
-        <f t="shared" si="0"/>
-        <v>2140001</v>
-      </c>
-      <c r="F6" t="str">
-        <f>A6&amp;B6&amp;C6</f>
-        <v>214</v>
-      </c>
-      <c r="G6" t="s">
-        <v>114</v>
-      </c>
-      <c r="H6" t="s">
-        <v>159</v>
-      </c>
-      <c r="I6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E7" t="str">
-        <f t="shared" si="0"/>
-        <v>2150001</v>
-      </c>
-      <c r="F7" t="str">
-        <f>A7&amp;B7&amp;C7</f>
-        <v>215</v>
-      </c>
-      <c r="G7" t="s">
-        <v>115</v>
-      </c>
-      <c r="H7" t="s">
-        <v>159</v>
-      </c>
-      <c r="I7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2</v>
-      </c>
-      <c r="B8">
-        <v>2</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E8" t="str">
-        <f t="shared" si="0"/>
-        <v>2210001</v>
-      </c>
-      <c r="F8" t="str">
-        <f>A8&amp;B8&amp;C8</f>
-        <v>221</v>
-      </c>
-      <c r="G8" t="s">
-        <v>117</v>
-      </c>
-      <c r="H8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I8" t="s">
-        <v>122</v>
+      <c r="H8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1860,40 +1875,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="A1" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
         <v>124</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>125</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>126</v>
       </c>
-      <c r="D2" t="s">
-        <v>127</v>
-      </c>
       <c r="E2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G2" t="s">
+        <v>149</v>
+      </c>
+      <c r="H2" t="s">
         <v>143</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" t="s">
         <v>148</v>
-      </c>
-      <c r="G2" t="s">
-        <v>150</v>
-      </c>
-      <c r="H2" t="s">
-        <v>144</v>
-      </c>
-      <c r="I2" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1907,7 +1922,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E3" t="str">
         <f>A3&amp;B3&amp;C3&amp;D3</f>
@@ -1918,10 +1933,10 @@
         <v>311</v>
       </c>
       <c r="G3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I3" t="s">
         <v>48</v>
@@ -1938,7 +1953,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" ref="E4:E8" si="0">A4&amp;B4&amp;C4&amp;D4</f>
@@ -1949,10 +1964,10 @@
         <v>312</v>
       </c>
       <c r="G4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I4" t="s">
         <v>48</v>
@@ -1969,7 +1984,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
@@ -1980,10 +1995,10 @@
         <v>313</v>
       </c>
       <c r="G5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I5" t="s">
         <v>48</v>
@@ -2000,7 +2015,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="0"/>
@@ -2011,10 +2026,10 @@
         <v>321</v>
       </c>
       <c r="G6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I6" t="s">
         <v>48</v>
@@ -2031,7 +2046,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="0"/>
@@ -2042,13 +2057,13 @@
         <v>322</v>
       </c>
       <c r="G7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H7" t="s">
         <v>48</v>
       </c>
       <c r="I7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -2062,7 +2077,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="0"/>
@@ -2073,10 +2088,10 @@
         <v>341</v>
       </c>
       <c r="G8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I8" t="s">
         <v>48</v>
@@ -2093,7 +2108,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" ref="E9" si="2">A9&amp;B9&amp;C9&amp;D9</f>
@@ -2104,10 +2119,10 @@
         <v>351</v>
       </c>
       <c r="G9" t="s">
+        <v>157</v>
+      </c>
+      <c r="H9" t="s">
         <v>158</v>
-      </c>
-      <c r="H9" t="s">
-        <v>159</v>
       </c>
       <c r="I9" t="s">
         <v>48</v>
@@ -2138,28 +2153,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="A1" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
         <v>124</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>125</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>126</v>
       </c>
-      <c r="D2" t="s">
-        <v>127</v>
-      </c>
       <c r="E2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -2173,7 +2188,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E3" t="str">
         <f>A3&amp;B3&amp;C3&amp;D3</f>
@@ -2191,7 +2206,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" ref="E4:E9" si="0">A4&amp;B4&amp;C4&amp;D4</f>
@@ -2209,7 +2224,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
@@ -2227,7 +2242,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="0"/>
@@ -2245,7 +2260,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="0"/>
@@ -2263,7 +2278,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="0"/>
@@ -2281,7 +2296,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="0"/>
@@ -2319,31 +2334,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="A1" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
         <v>124</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>125</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>126</v>
-      </c>
-      <c r="D2" t="s">
-        <v>127</v>
       </c>
       <c r="E2" t="s">
         <v>103</v>
       </c>
       <c r="F2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G2" t="s">
         <v>104</v>
@@ -2381,14 +2396,14 @@
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E3" t="str">
         <f>A3&amp;B3&amp;C3&amp;D3</f>
         <v>6110001</v>
       </c>
       <c r="F3" t="str">
-        <f>A3&amp;B3&amp;C3</f>
+        <f t="shared" ref="F3:F30" si="0">A3&amp;B3&amp;C3</f>
         <v>611</v>
       </c>
       <c r="G3" t="s">
@@ -2427,14 +2442,14 @@
         <v>1</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E4" t="str">
-        <f t="shared" ref="E4:E30" si="0">A4&amp;B4&amp;C4&amp;D4</f>
+        <f t="shared" ref="E4:E30" si="1">A4&amp;B4&amp;C4&amp;D4</f>
         <v>6110002</v>
       </c>
       <c r="F4" t="str">
-        <f>A4&amp;B4&amp;C4</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G4" t="s">
@@ -2473,14 +2488,14 @@
         <v>1</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110003</v>
       </c>
       <c r="F5" t="str">
-        <f>A5&amp;B5&amp;C5</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G5" t="s">
@@ -2519,14 +2534,14 @@
         <v>1</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110004</v>
       </c>
       <c r="F6" t="str">
-        <f>A6&amp;B6&amp;C6</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G6" t="s">
@@ -2565,14 +2580,14 @@
         <v>1</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E7" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110005</v>
       </c>
       <c r="F7" t="str">
-        <f>A7&amp;B7&amp;C7</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G7" t="s">
@@ -2611,14 +2626,14 @@
         <v>1</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E8" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110006</v>
       </c>
       <c r="F8" t="str">
-        <f>A8&amp;B8&amp;C8</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G8" t="s">
@@ -2657,14 +2672,14 @@
         <v>1</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E9" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110007</v>
       </c>
       <c r="F9" t="str">
-        <f>A9&amp;B9&amp;C9</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G9" t="s">
@@ -2703,14 +2718,14 @@
         <v>1</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E10" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110008</v>
       </c>
       <c r="F10" t="str">
-        <f>A10&amp;B10&amp;C10</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G10" t="s">
@@ -2749,14 +2764,14 @@
         <v>1</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E11" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110009</v>
       </c>
       <c r="F11" t="str">
-        <f>A11&amp;B11&amp;C11</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G11" t="s">
@@ -2795,14 +2810,14 @@
         <v>1</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E12" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110010</v>
       </c>
       <c r="F12" t="str">
-        <f>A12&amp;B12&amp;C12</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G12" t="s">
@@ -2841,14 +2856,14 @@
         <v>1</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110011</v>
       </c>
       <c r="F13" t="str">
-        <f>A13&amp;B13&amp;C13</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G13" t="s">
@@ -2887,14 +2902,14 @@
         <v>1</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110012</v>
       </c>
       <c r="F14" t="str">
-        <f>A14&amp;B14&amp;C14</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G14" t="s">
@@ -2933,14 +2948,14 @@
         <v>1</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110013</v>
       </c>
       <c r="F15" t="str">
-        <f>A15&amp;B15&amp;C15</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G15" t="s">
@@ -2979,14 +2994,14 @@
         <v>1</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E16" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6110014</v>
       </c>
       <c r="F16" t="str">
-        <f>A16&amp;B16&amp;C16</f>
+        <f t="shared" si="0"/>
         <v>611</v>
       </c>
       <c r="G16" t="s">
@@ -3025,14 +3040,14 @@
         <v>1</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6210001</v>
       </c>
       <c r="F17" t="str">
-        <f>A17&amp;B17&amp;C17</f>
+        <f t="shared" si="0"/>
         <v>621</v>
       </c>
       <c r="G17" s="1" t="s">
@@ -3068,14 +3083,14 @@
         <v>1</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E18" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6210002</v>
       </c>
       <c r="F18" t="str">
-        <f>A18&amp;B18&amp;C18</f>
+        <f t="shared" si="0"/>
         <v>621</v>
       </c>
       <c r="G18" s="1" t="s">
@@ -3111,14 +3126,14 @@
         <v>1</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E19" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6210003</v>
       </c>
       <c r="F19" t="str">
-        <f>A19&amp;B19&amp;C19</f>
+        <f t="shared" si="0"/>
         <v>621</v>
       </c>
       <c r="G19" s="1" t="s">
@@ -3154,14 +3169,14 @@
         <v>2</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6220001</v>
       </c>
       <c r="F20" t="str">
-        <f>A20&amp;B20&amp;C20</f>
+        <f t="shared" si="0"/>
         <v>622</v>
       </c>
       <c r="G20" s="1" t="s">
@@ -3197,14 +3212,14 @@
         <v>2</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E21" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6220002</v>
       </c>
       <c r="F21" t="str">
-        <f>A21&amp;B21&amp;C21</f>
+        <f t="shared" si="0"/>
         <v>622</v>
       </c>
       <c r="G21" s="1" t="s">
@@ -3240,14 +3255,14 @@
         <v>2</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6220003</v>
       </c>
       <c r="F22" t="str">
-        <f>A22&amp;B22&amp;C22</f>
+        <f t="shared" si="0"/>
         <v>622</v>
       </c>
       <c r="G22" s="1" t="s">
@@ -3283,14 +3298,14 @@
         <v>2</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6220004</v>
       </c>
       <c r="F23" t="str">
-        <f>A23&amp;B23&amp;C23</f>
+        <f t="shared" si="0"/>
         <v>622</v>
       </c>
       <c r="G23" s="1" t="s">
@@ -3326,14 +3341,14 @@
         <v>2</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6220005</v>
       </c>
       <c r="F24" t="str">
-        <f>A24&amp;B24&amp;C24</f>
+        <f t="shared" si="0"/>
         <v>622</v>
       </c>
       <c r="G24" s="1" t="s">
@@ -3369,14 +3384,14 @@
         <v>3</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6230001</v>
       </c>
       <c r="F25" t="str">
-        <f>A25&amp;B25&amp;C25</f>
+        <f t="shared" si="0"/>
         <v>623</v>
       </c>
       <c r="G25" s="1" t="s">
@@ -3412,14 +3427,14 @@
         <v>1</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E26" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6310001</v>
       </c>
       <c r="F26" t="str">
-        <f>A26&amp;B26&amp;C26</f>
+        <f t="shared" si="0"/>
         <v>631</v>
       </c>
       <c r="G26" s="1" t="s">
@@ -3455,14 +3470,14 @@
         <v>1</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6310002</v>
       </c>
       <c r="F27" t="str">
-        <f>A27&amp;B27&amp;C27</f>
+        <f t="shared" si="0"/>
         <v>631</v>
       </c>
       <c r="G27" s="1" t="s">
@@ -3498,14 +3513,14 @@
         <v>1</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E28" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6310003</v>
       </c>
       <c r="F28" t="str">
-        <f>A28&amp;B28&amp;C28</f>
+        <f t="shared" si="0"/>
         <v>631</v>
       </c>
       <c r="G28" s="1" t="s">
@@ -3541,14 +3556,14 @@
         <v>1</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E29" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6410001</v>
       </c>
       <c r="F29" t="str">
-        <f>A29&amp;B29&amp;C29</f>
+        <f t="shared" si="0"/>
         <v>641</v>
       </c>
       <c r="G29" t="s">
@@ -3584,14 +3599,14 @@
         <v>1</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E30" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6410002</v>
       </c>
       <c r="F30" t="str">
-        <f>A30&amp;B30&amp;C30</f>
+        <f t="shared" si="0"/>
         <v>641</v>
       </c>
       <c r="G30" t="s">

</xml_diff>